<commit_message>
Add equivalent cylinder and Starship example
</commit_message>
<xml_diff>
--- a/input_template.xlsx
+++ b/input_template.xlsx
@@ -1055,31 +1055,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V3"/>
+  <dimension ref="A1:Y3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
     <col width="6" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="7" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="7" customWidth="1" min="12" max="12"/>
-    <col width="7" customWidth="1" min="13" max="13"/>
-    <col width="8" customWidth="1" min="14" max="14"/>
-    <col width="8" customWidth="1" min="15" max="15"/>
-    <col width="8" customWidth="1" min="16" max="16"/>
-    <col width="6" customWidth="1" min="17" max="17"/>
-    <col width="5" customWidth="1" min="18" max="18"/>
-    <col width="7" customWidth="1" min="19" max="19"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="7" customWidth="1" min="16" max="16"/>
+    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
     <col width="6" customWidth="1" min="20" max="20"/>
-    <col width="7" customWidth="1" min="21" max="21"/>
-    <col width="4" customWidth="1" min="22" max="22"/>
+    <col width="5" customWidth="1" min="21" max="21"/>
+    <col width="7" customWidth="1" min="22" max="22"/>
+    <col width="6" customWidth="1" min="23" max="23"/>
+    <col width="7" customWidth="1" min="24" max="24"/>
+    <col width="4" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1105,90 +1108,105 @@
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
+          <t>几何类型</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>等效半径R</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>等效高度H</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
           <t>推进剂密度rho_phi</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>气体密度rho_g</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>秒流量mdot</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>加注量Mf</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>关机剩余量Mr</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>启动后剩余量Mef</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>坐标原点X或Loki</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>坐标原点Y</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>坐标原点Z</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="Q1" s="2" t="inlineStr">
         <is>
           <t>点火时间tf</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="R1" s="2" t="inlineStr">
         <is>
           <t>关机时间tb</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="S1" s="2" t="inlineStr">
         <is>
           <t>分离时间ts</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="T1" s="2" t="inlineStr">
         <is>
           <t>箱底hb</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="U1" s="2" t="inlineStr">
         <is>
           <t>总高H</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="V1" s="2" t="inlineStr">
         <is>
           <t>总容积Vo</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="W1" s="2" t="inlineStr">
         <is>
           <t>满箱Xo</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="X1" s="2" t="inlineStr">
         <is>
           <t>满箱Jyo</t>
         </is>
       </c>
-      <c r="V1" s="2" t="inlineStr">
+      <c r="Y1" s="2" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -1211,58 +1229,69 @@
           <t>一级氧化剂箱</t>
         </is>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>等效圆柱</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H2" s="3" t="n">
         <v>1140</v>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="I2" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="J2" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="H2" s="3" t="n">
+      <c r="K2" s="3" t="n">
         <v>6000</v>
       </c>
-      <c r="I2" s="3" t="n">
+      <c r="L2" s="3" t="n">
         <v>300</v>
       </c>
-      <c r="J2" s="3" t="n">
+      <c r="M2" s="3" t="n">
         <v>6000</v>
       </c>
-      <c r="K2" s="3" t="n">
+      <c r="N2" s="3" t="n">
         <v>45</v>
       </c>
-      <c r="L2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" s="3" t="n">
-        <v>0</v>
-      </c>
       <c r="O2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" s="3" t="n">
         <v>120</v>
       </c>
-      <c r="P2" s="3" t="n">
+      <c r="S2" s="3" t="n">
         <v>125</v>
       </c>
-      <c r="Q2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="S2" s="3" t="n">
-        <v>5.3</v>
-      </c>
       <c r="T2" s="3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="U2" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="V2" s="3" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="W2" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="X2" s="3" t="n">
         <v>90000</v>
       </c>
-      <c r="V2" s="3" t="inlineStr">
+      <c r="Y2" s="3" t="inlineStr">
         <is>
           <t>示例</t>
         </is>
@@ -1285,58 +1314,69 @@
           <t>一级燃料箱</t>
         </is>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>等效圆柱</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="H3" s="3" t="n">
         <v>810</v>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="I3" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G3" s="3" t="n">
+      <c r="J3" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="H3" s="3" t="n">
+      <c r="K3" s="3" t="n">
         <v>3500</v>
       </c>
-      <c r="I3" s="3" t="n">
+      <c r="L3" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="J3" s="3" t="n">
+      <c r="M3" s="3" t="n">
         <v>3500</v>
       </c>
-      <c r="K3" s="3" t="n">
+      <c r="N3" s="3" t="n">
         <v>32</v>
       </c>
-      <c r="L3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" s="3" t="n">
-        <v>0</v>
-      </c>
       <c r="O3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" s="3" t="n">
         <v>120</v>
       </c>
-      <c r="P3" s="3" t="n">
+      <c r="S3" s="3" t="n">
         <v>125</v>
       </c>
-      <c r="Q3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="S3" s="3" t="n">
-        <v>4.3</v>
-      </c>
       <c r="T3" s="3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U3" s="3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="V3" s="3" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="W3" s="3" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="X3" s="3" t="n">
         <v>50000</v>
       </c>
-      <c r="V3" s="3" t="inlineStr">
+      <c r="Y3" s="3" t="inlineStr">
         <is>
           <t>示例</t>
         </is>

</xml_diff>